<commit_message>
Changed board creation system
</commit_message>
<xml_diff>
--- a/Docs/Abilities.xlsx
+++ b/Docs/Abilities.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="223">
   <si>
     <t>Name</t>
   </si>
@@ -618,9 +618,6 @@
     <t>""who needs attention</t>
   </si>
   <si>
-    <t>This unit's attack damage is always equal to the number of nearby cells occupied by friendly units</t>
-  </si>
-  <si>
     <t>Ratbearer</t>
   </si>
   <si>
@@ -676,6 +673,18 @@
   </si>
   <si>
     <t>After deploying this unit, you can select another unit with "Cheap" to be deployed</t>
+  </si>
+  <si>
+    <t>Lethal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This unit's attack damage is equal to the total amount of attack damage between all friendly units within 1 cell </t>
+  </si>
+  <si>
+    <t>lethal ""</t>
+  </si>
+  <si>
+    <t>All succesfull attack damage dealt instantly destroys the target</t>
   </si>
 </sst>
 </file>
@@ -1209,7 +1218,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J142"/>
+  <dimension ref="A1:J147"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.140625" style="3" customWidth="1"/>
@@ -1353,7 +1362,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>0</v>
@@ -1376,7 +1385,7 @@
         <v>84</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>84</v>
@@ -1536,7 +1545,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>0</v>
@@ -1576,7 +1585,7 @@
         <v>84</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>84</v>
@@ -1856,7 +1865,7 @@
         <v>0</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I39" s="4" t="s">
         <v>0</v>
@@ -1916,7 +1925,7 @@
         <v>6</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="I42" s="4" t="s">
         <v>6</v>
@@ -1936,7 +1945,7 @@
         <v>0</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>0</v>
@@ -1996,7 +2005,7 @@
         <v>6</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I47" s="8" t="s">
         <v>6</v>
@@ -2098,7 +2107,7 @@
         <v>0</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F54" s="8" t="s">
         <v>68</v>
@@ -2312,7 +2321,7 @@
         <v>6</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="I67" s="4" t="s">
         <v>6</v>
@@ -2392,7 +2401,7 @@
         <v>6</v>
       </c>
       <c r="G72" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I72" s="8" t="s">
         <v>6</v>
@@ -3154,7 +3163,7 @@
         <v>0</v>
       </c>
       <c r="D134" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F134" s="4" t="s">
         <v>0</v>
@@ -3174,7 +3183,7 @@
         <v>99</v>
       </c>
       <c r="D135" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F135" s="4" t="s">
         <v>99</v>
@@ -3214,7 +3223,7 @@
         <v>6</v>
       </c>
       <c r="D137" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F137" s="4" t="s">
         <v>6</v>
@@ -3230,11 +3239,11 @@
       </c>
     </row>
     <row r="139" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C139" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="D139" s="7" t="s">
-        <v>212</v>
+      <c r="C139" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D139" s="8" t="s">
+        <v>211</v>
       </c>
       <c r="F139" s="7" t="s">
         <v>0</v>
@@ -3246,15 +3255,15 @@
         <v>0</v>
       </c>
       <c r="J139" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="140" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C140" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="D140" s="7" t="s">
-        <v>213</v>
+      <c r="C140" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="D140" s="8" t="s">
+        <v>212</v>
       </c>
       <c r="F140" s="7" t="s">
         <v>99</v>
@@ -3270,10 +3279,10 @@
       </c>
     </row>
     <row r="141" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C141" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D141" s="7" t="s">
+      <c r="C141" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D141" s="8" t="s">
         <v>12</v>
       </c>
       <c r="F141" s="7" t="s">
@@ -3290,23 +3299,55 @@
       </c>
     </row>
     <row r="142" spans="3:10" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C142" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D142" s="7" t="s">
+      <c r="C142" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D142" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="F142" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G142" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="I142" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J142" s="4" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="144" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C144" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="D144" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="F142" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="G142" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="I142" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J142" s="4" t="s">
-        <v>211</v>
+    </row>
+    <row r="145" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C145" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D145" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="146" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C146" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D146" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="147" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C147" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D147" s="7" t="s">
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>